<commit_message>
release 220 (#432) 398f54831a4af027755f06dfb895bf3122858145
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-tddui-discriminator.xlsx
+++ b/main/ig/CodeSystem-tddui-discriminator.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.2.0-ballot</t>
+    <t>2.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-05T15:15:02+00:00</t>
+    <t>2026-02-06T13:40:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publi 230 (#457) c79d080acbcd6771416f83bcf76893d7f235d5bd
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-tddui-discriminator.xlsx
+++ b/main/ig/CodeSystem-tddui-discriminator.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.3.0-ballot</t>
+    <t>2.3.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-02T11:00:56+00:00</t>
+    <t>2026-03-16T15:16:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>